<commit_message>
feat: script migracion mejorado para identificar correctamente WFS con formato de salida json compatible con arcgis, gml xml no lo son
</commit_message>
<xml_diff>
--- a/data/inventario_fuentes_app.xlsx
+++ b/data/inventario_fuentes_app.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30117"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UPNA\Practicas\Proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B823162-BA3D-443D-ACC7-6D853EF4FD1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2031" documentId="11_AA6545BBAF73DF827D66C660FEB33D2A0657F1FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08AAA5C9-5DC0-4E17-9244-B38835B327C2}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,8 +21,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">inventario_fuentes_GIS_v2!$A$122:$A$122</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">inventario_fuentes_GIS!$AB$1:$AB$132</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Referencias!$B$14:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">inventario_fuentes_GIS!$S$139:$S$139</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -80,7 +80,7 @@
     <t>requiere_registro</t>
   </si>
   <si>
-    <t>fomato_datos</t>
+    <t>formato_datos</t>
   </si>
   <si>
     <t>tematica_inspire</t>
@@ -1104,7 +1104,7 @@
     <t>https://www.ign.es/wfs/redes-geodesicas</t>
   </si>
   <si>
-    <t>RECORTE</t>
+    <t>GML / XML/application/json</t>
   </si>
   <si>
     <t>Coordinate Reference Systems - RS / Geographical Grid Systems - GG</t>
@@ -3913,6 +3913,9 @@
     <t>El servicio permite consumir datos delimitando una caja geográfica (Bounding Box) que cubra el área de interés.</t>
   </si>
   <si>
+    <t>RECORTE</t>
+  </si>
+  <si>
     <t>Requiere la descarga del conjunto de datos completo para su posterior recorte mediante el límite municipal oficial.</t>
   </si>
   <si>
@@ -3944,9 +3947,6 @@
   </si>
   <si>
     <t>Modelo basado en el consumo de recursos (pay-as-you-go) mediante claves de autenticación.</t>
-  </si>
-  <si>
-    <t>formato_datos</t>
   </si>
   <si>
     <t>Servicio Raster: Entrega imágenes dinámicas; ideal para visualización pero limitado para análisis de datos crudos.</t>
@@ -4139,7 +4139,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4333,6 +4333,13 @@
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="36">
@@ -4695,7 +4702,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
@@ -4725,6 +4732,7 @@
     <xf numFmtId="0" fontId="22" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -5208,37 +5216,15 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DEEA9DB5-F116-421D-B567-A40619913A8C}" name="Tabla14" displayName="Tabla14" ref="A1:X132" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A1:X132" xr:uid="{3167EED3-35A1-4778-BDE4-B1E5EDFBDC62}">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
-    <filterColumn colId="7" hiddenButton="1"/>
-    <filterColumn colId="8" hiddenButton="1"/>
-    <filterColumn colId="9" hiddenButton="1"/>
-    <filterColumn colId="10" hiddenButton="1"/>
-    <filterColumn colId="11" hiddenButton="1"/>
-    <filterColumn colId="12" hiddenButton="1"/>
-    <filterColumn colId="13" hiddenButton="1"/>
-    <filterColumn colId="14" hiddenButton="1"/>
-    <filterColumn colId="15" hiddenButton="1"/>
-    <filterColumn colId="16" hiddenButton="1"/>
-    <filterColumn colId="17" hiddenButton="1"/>
-    <filterColumn colId="18" hiddenButton="1"/>
-    <filterColumn colId="19" hiddenButton="1"/>
-    <filterColumn colId="20" hiddenButton="1"/>
-    <filterColumn colId="21" hiddenButton="1"/>
-    <filterColumn colId="22" hiddenButton="1"/>
-    <filterColumn colId="23" hiddenButton="1"/>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="OGC WFS"/>
+        <filter val="OGC WFS / WFS INSPIRE"/>
+        <filter val="WFS"/>
+        <filter val="WFS / Descarga directa"/>
+      </filters>
+    </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:W132">
-    <sortCondition ref="A2:A132"/>
-    <sortCondition descending="1" ref="T2:T132"/>
-    <sortCondition ref="B2:B132"/>
-    <sortCondition ref="C2:C132"/>
-  </sortState>
   <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{F1C31A27-0811-4E1A-B500-1B4FE61DDF79}" name="bloque_tematico" dataDxfId="36"/>
     <tableColumn id="2" xr3:uid="{1C1A8726-C54C-4252-9546-FFA9EEEEEF7B}" name="subtema" dataDxfId="35"/>
@@ -5251,7 +5237,7 @@
     <tableColumn id="14" xr3:uid="{DB7B7FDF-DB75-4F19-ABE8-2FB051EEFFB3}" name="disponibilidad_municipal"/>
     <tableColumn id="9" xr3:uid="{FC78D287-D099-4DF4-A13E-28E2C1B881A6}" name="coste" dataDxfId="29"/>
     <tableColumn id="10" xr3:uid="{E8B3B73B-B302-4FB2-8D9C-E9644AB28FEE}" name="requiere_registro" dataDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{06B0F86C-3DA0-4159-80B8-8C8978F397A1}" name="fomato_datos" dataDxfId="27"/>
+    <tableColumn id="11" xr3:uid="{06B0F86C-3DA0-4159-80B8-8C8978F397A1}" name="formato_datos" dataDxfId="27"/>
     <tableColumn id="12" xr3:uid="{FAA8B6CC-31C2-41C9-8146-AAF380258AA7}" name="tematica_inspire" dataDxfId="26"/>
     <tableColumn id="13" xr3:uid="{AA85804C-1FE8-49B8-8A96-32779C75E905}" name="notas_limitaciones" dataDxfId="25"/>
     <tableColumn id="17" xr3:uid="{CB16B685-F8D5-4BAB-AB25-1A8B191039F5}" name="capabilities" dataDxfId="24"/>
@@ -5590,7 +5576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ABDB362-2FA5-4E80-8780-2B0AEA417E8C}">
-  <dimension ref="A1:AF128"/>
+  <dimension ref="A1:AF132"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.42578125" bestFit="1" customWidth="1"/>
@@ -5606,7 +5592,7 @@
     <col min="12" max="12" width="25.85546875" customWidth="1"/>
     <col min="13" max="13" width="45.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="55.42578125" customWidth="1"/>
-    <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="15" max="15" width="37.7109375" customWidth="1"/>
     <col min="16" max="21" width="16.42578125" customWidth="1"/>
     <col min="22" max="22" width="35.5703125" customWidth="1"/>
     <col min="23" max="23" width="16.42578125" customWidth="1"/>
@@ -5687,7 +5673,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" spans="1:26" hidden="1">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -5802,7 +5788,7 @@
       <c r="N3" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="1" t="s">
         <v>45</v>
       </c>
       <c r="P3" s="7">
@@ -5895,7 +5881,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:26" hidden="1">
       <c r="A5" s="7" t="s">
         <v>24</v>
       </c>
@@ -5955,7 +5941,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:26">
+    <row r="6" spans="1:26" hidden="1">
       <c r="A6" s="7" t="s">
         <v>66</v>
       </c>
@@ -6027,7 +6013,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:26">
+    <row r="7" spans="1:26" hidden="1">
       <c r="A7" s="7" t="s">
         <v>66</v>
       </c>
@@ -6099,7 +6085,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:26">
+    <row r="8" spans="1:26" hidden="1">
       <c r="A8" s="7" t="s">
         <v>66</v>
       </c>
@@ -6171,7 +6157,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:26">
+    <row r="9" spans="1:26" hidden="1">
       <c r="A9" s="7" t="s">
         <v>66</v>
       </c>
@@ -6243,7 +6229,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="10" spans="1:26">
+    <row r="10" spans="1:26" hidden="1">
       <c r="A10" s="7" t="s">
         <v>66</v>
       </c>
@@ -6315,7 +6301,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:26">
+    <row r="11" spans="1:26" hidden="1">
       <c r="A11" s="7" t="s">
         <v>66</v>
       </c>
@@ -6387,7 +6373,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="12" spans="1:26">
+    <row r="12" spans="1:26" hidden="1">
       <c r="A12" s="7" t="s">
         <v>66</v>
       </c>
@@ -6459,7 +6445,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:26">
+    <row r="13" spans="1:26" hidden="1">
       <c r="A13" s="7" t="s">
         <v>66</v>
       </c>
@@ -6531,7 +6517,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:26">
+    <row r="14" spans="1:26" hidden="1">
       <c r="A14" s="7" t="s">
         <v>66</v>
       </c>
@@ -6603,7 +6589,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="1:26">
+    <row r="15" spans="1:26" hidden="1">
       <c r="A15" s="7" t="s">
         <v>66</v>
       </c>
@@ -6675,7 +6661,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:26">
+    <row r="16" spans="1:26" hidden="1">
       <c r="A16" s="7" t="s">
         <v>66</v>
       </c>
@@ -6747,7 +6733,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="17" spans="1:24">
+    <row r="17" spans="1:24" hidden="1">
       <c r="A17" s="7" t="s">
         <v>66</v>
       </c>
@@ -6819,7 +6805,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:24">
+    <row r="18" spans="1:24" hidden="1">
       <c r="A18" s="7" t="s">
         <v>66</v>
       </c>
@@ -6891,7 +6877,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:24">
+    <row r="19" spans="1:24" hidden="1">
       <c r="A19" s="7" t="s">
         <v>66</v>
       </c>
@@ -6963,7 +6949,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:24">
+    <row r="20" spans="1:24" hidden="1">
       <c r="A20" s="7" t="s">
         <v>66</v>
       </c>
@@ -7035,7 +7021,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="21" spans="1:24">
+    <row r="21" spans="1:24" hidden="1">
       <c r="A21" s="7" t="s">
         <v>66</v>
       </c>
@@ -7107,7 +7093,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="22" spans="1:24">
+    <row r="22" spans="1:24" hidden="1">
       <c r="A22" s="7" t="s">
         <v>66</v>
       </c>
@@ -7179,7 +7165,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:24">
+    <row r="23" spans="1:24" hidden="1">
       <c r="A23" s="7" t="s">
         <v>66</v>
       </c>
@@ -7251,7 +7237,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:24">
+    <row r="24" spans="1:24" hidden="1">
       <c r="A24" s="7" t="s">
         <v>66</v>
       </c>
@@ -7323,7 +7309,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="1:24">
+    <row r="25" spans="1:24" hidden="1">
       <c r="A25" s="7" t="s">
         <v>66</v>
       </c>
@@ -7395,7 +7381,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="26" spans="1:24">
+    <row r="26" spans="1:24" hidden="1">
       <c r="A26" s="7" t="s">
         <v>66</v>
       </c>
@@ -7467,7 +7453,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="27" spans="1:24">
+    <row r="27" spans="1:24" hidden="1">
       <c r="A27" s="7" t="s">
         <v>66</v>
       </c>
@@ -7539,7 +7525,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="28" spans="1:24">
+    <row r="28" spans="1:24" hidden="1">
       <c r="A28" s="7" t="s">
         <v>66</v>
       </c>
@@ -7611,7 +7597,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="29" spans="1:24">
+    <row r="29" spans="1:24" hidden="1">
       <c r="A29" s="7" t="s">
         <v>66</v>
       </c>
@@ -7683,7 +7669,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="30" spans="1:24">
+    <row r="30" spans="1:24" hidden="1">
       <c r="A30" s="7" t="s">
         <v>66</v>
       </c>
@@ -7755,7 +7741,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="31" spans="1:24">
+    <row r="31" spans="1:24" hidden="1">
       <c r="A31" s="7" t="s">
         <v>66</v>
       </c>
@@ -7827,7 +7813,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="32" spans="1:24">
+    <row r="32" spans="1:24" hidden="1">
       <c r="A32" s="7" t="s">
         <v>66</v>
       </c>
@@ -7899,7 +7885,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="33" spans="1:24">
+    <row r="33" spans="1:24" hidden="1">
       <c r="A33" s="7" t="s">
         <v>66</v>
       </c>
@@ -7971,7 +7957,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="34" spans="1:24">
+    <row r="34" spans="1:24" hidden="1">
       <c r="A34" s="7" t="s">
         <v>66</v>
       </c>
@@ -8043,7 +8029,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="35" spans="1:24">
+    <row r="35" spans="1:24" hidden="1">
       <c r="A35" s="7" t="s">
         <v>66</v>
       </c>
@@ -8115,7 +8101,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="1:24">
+    <row r="36" spans="1:24" hidden="1">
       <c r="A36" s="7" t="s">
         <v>66</v>
       </c>
@@ -8126,7 +8112,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="37" spans="1:24">
+    <row r="37" spans="1:24" hidden="1">
       <c r="A37" t="s">
         <v>232</v>
       </c>
@@ -8198,7 +8184,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="38" spans="1:24">
+    <row r="38" spans="1:24" hidden="1">
       <c r="A38" t="s">
         <v>232</v>
       </c>
@@ -8269,7 +8255,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="39" spans="1:24">
+    <row r="39" spans="1:24" hidden="1">
       <c r="A39" t="s">
         <v>232</v>
       </c>
@@ -8340,7 +8326,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="40" spans="1:24">
+    <row r="40" spans="1:24" hidden="1">
       <c r="A40" t="s">
         <v>232</v>
       </c>
@@ -8412,7 +8398,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="41" spans="1:24">
+    <row r="41" spans="1:24" hidden="1">
       <c r="A41" t="s">
         <v>232</v>
       </c>
@@ -8484,7 +8470,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="42" spans="1:24">
+    <row r="42" spans="1:24" hidden="1">
       <c r="A42" t="s">
         <v>232</v>
       </c>
@@ -8556,7 +8542,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="43" spans="1:24">
+    <row r="43" spans="1:24" hidden="1">
       <c r="A43" t="s">
         <v>232</v>
       </c>
@@ -8627,7 +8613,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="44" spans="1:24">
+    <row r="44" spans="1:24" hidden="1">
       <c r="A44" t="s">
         <v>232</v>
       </c>
@@ -8699,7 +8685,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="45" spans="1:24">
+    <row r="45" spans="1:24" hidden="1">
       <c r="A45" t="s">
         <v>232</v>
       </c>
@@ -8771,7 +8757,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="46" spans="1:24">
+    <row r="46" spans="1:24" hidden="1">
       <c r="A46" t="s">
         <v>232</v>
       </c>
@@ -8843,7 +8829,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="47" spans="1:24">
+    <row r="47" spans="1:24" hidden="1">
       <c r="A47" t="s">
         <v>232</v>
       </c>
@@ -8915,7 +8901,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="48" spans="1:24">
+    <row r="48" spans="1:24" hidden="1">
       <c r="A48" t="s">
         <v>232</v>
       </c>
@@ -8987,7 +8973,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="49" spans="1:24">
+    <row r="49" spans="1:24" hidden="1">
       <c r="A49" t="s">
         <v>232</v>
       </c>
@@ -9058,7 +9044,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="50" spans="1:24">
+    <row r="50" spans="1:24" hidden="1">
       <c r="A50" t="s">
         <v>232</v>
       </c>
@@ -9129,7 +9115,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="51" spans="1:24">
+    <row r="51" spans="1:24" hidden="1">
       <c r="A51" t="s">
         <v>232</v>
       </c>
@@ -9201,7 +9187,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="52" spans="1:24">
+    <row r="52" spans="1:24" hidden="1">
       <c r="A52" t="s">
         <v>232</v>
       </c>
@@ -9273,7 +9259,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="53" spans="1:24">
+    <row r="53" spans="1:24" hidden="1">
       <c r="A53" t="s">
         <v>232</v>
       </c>
@@ -9369,7 +9355,7 @@
       </c>
       <c r="H54" s="7"/>
       <c r="I54" s="7" t="s">
-        <v>347</v>
+        <v>31</v>
       </c>
       <c r="J54" s="7" t="s">
         <v>32</v>
@@ -9378,7 +9364,7 @@
         <v>33</v>
       </c>
       <c r="L54" s="7" t="s">
-        <v>51</v>
+        <v>347</v>
       </c>
       <c r="M54" s="7" t="s">
         <v>348</v>
@@ -9386,7 +9372,7 @@
       <c r="N54" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="O54" s="7" t="s">
+      <c r="O54" s="1" t="s">
         <v>350</v>
       </c>
       <c r="P54" s="7">
@@ -9417,7 +9403,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="55" spans="1:24">
+    <row r="55" spans="1:24" hidden="1">
       <c r="A55" t="s">
         <v>232</v>
       </c>
@@ -9488,7 +9474,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="56" spans="1:24">
+    <row r="56" spans="1:24" hidden="1">
       <c r="A56" t="s">
         <v>232</v>
       </c>
@@ -9560,7 +9546,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="57" spans="1:24">
+    <row r="57" spans="1:24" hidden="1">
       <c r="A57" t="s">
         <v>232</v>
       </c>
@@ -9632,7 +9618,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="58" spans="1:24">
+    <row r="58" spans="1:24" hidden="1">
       <c r="A58" t="s">
         <v>232</v>
       </c>
@@ -9704,7 +9690,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="59" spans="1:24">
+    <row r="59" spans="1:24" hidden="1">
       <c r="A59" t="s">
         <v>232</v>
       </c>
@@ -9776,7 +9762,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="60" spans="1:24">
+    <row r="60" spans="1:24" hidden="1">
       <c r="A60" t="s">
         <v>232</v>
       </c>
@@ -9848,7 +9834,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="61" spans="1:24">
+    <row r="61" spans="1:24" hidden="1">
       <c r="A61" t="s">
         <v>232</v>
       </c>
@@ -9920,7 +9906,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="62" spans="1:24">
+    <row r="62" spans="1:24" hidden="1">
       <c r="A62" s="7" t="s">
         <v>232</v>
       </c>
@@ -9992,7 +9978,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="63" spans="1:24">
+    <row r="63" spans="1:24" hidden="1">
       <c r="A63" t="s">
         <v>232</v>
       </c>
@@ -10064,7 +10050,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="64" spans="1:24">
+    <row r="64" spans="1:24" hidden="1">
       <c r="A64" t="s">
         <v>232</v>
       </c>
@@ -10136,7 +10122,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="65" spans="1:24">
+    <row r="65" spans="1:24" hidden="1">
       <c r="A65" t="s">
         <v>232</v>
       </c>
@@ -10208,7 +10194,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="66" spans="1:24">
+    <row r="66" spans="1:24" hidden="1">
       <c r="A66" t="s">
         <v>232</v>
       </c>
@@ -10280,7 +10266,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:24">
+    <row r="67" spans="1:24" hidden="1">
       <c r="A67" t="s">
         <v>232</v>
       </c>
@@ -10352,7 +10338,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="68" spans="1:24">
+    <row r="68" spans="1:24" hidden="1">
       <c r="A68" t="s">
         <v>232</v>
       </c>
@@ -10424,7 +10410,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="69" spans="1:24">
+    <row r="69" spans="1:24" hidden="1">
       <c r="A69" t="s">
         <v>232</v>
       </c>
@@ -10498,7 +10484,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="70" spans="1:24">
+    <row r="70" spans="1:24" hidden="1">
       <c r="A70" t="s">
         <v>232</v>
       </c>
@@ -10604,7 +10590,7 @@
       <c r="K71" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="L71" s="7" t="s">
+      <c r="L71" s="19" t="s">
         <v>451</v>
       </c>
       <c r="M71" s="7" t="s">
@@ -10685,7 +10671,7 @@
       <c r="N72" s="7" t="s">
         <v>458</v>
       </c>
-      <c r="O72" s="7" t="s">
+      <c r="O72" s="1" t="s">
         <v>459</v>
       </c>
       <c r="P72" s="7">
@@ -10716,7 +10702,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="73" spans="1:24">
+    <row r="73" spans="1:24" hidden="1">
       <c r="A73" s="7" t="s">
         <v>445</v>
       </c>
@@ -10928,7 +10914,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="76" spans="1:24">
+    <row r="76" spans="1:24" hidden="1">
       <c r="A76" s="7" t="s">
         <v>445</v>
       </c>
@@ -10998,7 +10984,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="77" spans="1:24">
+    <row r="77" spans="1:24" hidden="1">
       <c r="A77" s="7" t="s">
         <v>445</v>
       </c>
@@ -11070,7 +11056,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:24">
+    <row r="78" spans="1:24" hidden="1">
       <c r="A78" s="7" t="s">
         <v>445</v>
       </c>
@@ -11139,7 +11125,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="79" spans="1:24">
+    <row r="79" spans="1:24" hidden="1">
       <c r="A79" s="7" t="s">
         <v>496</v>
       </c>
@@ -11211,7 +11197,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="80" spans="1:24">
+    <row r="80" spans="1:24" hidden="1">
       <c r="A80" s="7" t="s">
         <v>496</v>
       </c>
@@ -11294,7 +11280,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="82" spans="1:24">
+    <row r="82" spans="1:24" hidden="1">
       <c r="A82" s="7" t="s">
         <v>509</v>
       </c>
@@ -11366,7 +11352,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="83" spans="1:24">
+    <row r="83" spans="1:24" hidden="1">
       <c r="A83" s="7" t="s">
         <v>530</v>
       </c>
@@ -11377,7 +11363,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="84" spans="1:24">
+    <row r="84" spans="1:24" hidden="1">
       <c r="A84" t="s">
         <v>532</v>
       </c>
@@ -11449,7 +11435,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="85" spans="1:24">
+    <row r="85" spans="1:24" hidden="1">
       <c r="A85" s="7" t="s">
         <v>540</v>
       </c>
@@ -11460,7 +11446,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="86" spans="1:24">
+    <row r="86" spans="1:24" hidden="1">
       <c r="A86" s="7" t="s">
         <v>540</v>
       </c>
@@ -11471,7 +11457,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="87" spans="1:24">
+    <row r="87" spans="1:24" hidden="1">
       <c r="A87" s="7" t="s">
         <v>543</v>
       </c>
@@ -11615,7 +11601,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="89" spans="1:24">
+    <row r="89" spans="1:24" hidden="1">
       <c r="A89" s="7" t="s">
         <v>550</v>
       </c>
@@ -11687,7 +11673,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="90" spans="1:24">
+    <row r="90" spans="1:24" hidden="1">
       <c r="A90" s="7" t="s">
         <v>550</v>
       </c>
@@ -11759,7 +11745,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="91" spans="1:24">
+    <row r="91" spans="1:24" hidden="1">
       <c r="A91" s="7" t="s">
         <v>550</v>
       </c>
@@ -11831,7 +11817,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="92" spans="1:24">
+    <row r="92" spans="1:24" hidden="1">
       <c r="A92" s="7" t="s">
         <v>550</v>
       </c>
@@ -11842,7 +11828,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="93" spans="1:24">
+    <row r="93" spans="1:24" hidden="1">
       <c r="A93" s="7" t="s">
         <v>550</v>
       </c>
@@ -11853,7 +11839,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="94" spans="1:24">
+    <row r="94" spans="1:24" hidden="1">
       <c r="A94" t="s">
         <v>580</v>
       </c>
@@ -11918,7 +11904,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="95" spans="1:24">
+    <row r="95" spans="1:24" hidden="1">
       <c r="A95" t="s">
         <v>580</v>
       </c>
@@ -11986,7 +11972,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="96" spans="1:24">
+    <row r="96" spans="1:24" hidden="1">
       <c r="A96" t="s">
         <v>580</v>
       </c>
@@ -12054,7 +12040,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="97" spans="1:24" ht="15" customHeight="1">
+    <row r="97" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A97" t="s">
         <v>580</v>
       </c>
@@ -12122,7 +12108,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="98" spans="1:24" ht="15" customHeight="1">
+    <row r="98" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A98" t="s">
         <v>580</v>
       </c>
@@ -12190,7 +12176,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="99" spans="1:24" ht="15" customHeight="1">
+    <row r="99" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A99" t="s">
         <v>580</v>
       </c>
@@ -12246,7 +12232,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="100" spans="1:24" ht="15" customHeight="1">
+    <row r="100" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A100" t="s">
         <v>580</v>
       </c>
@@ -12302,7 +12288,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="101" spans="1:24" ht="15" customHeight="1">
+    <row r="101" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A101" t="s">
         <v>580</v>
       </c>
@@ -12358,7 +12344,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="102" spans="1:24" ht="15" customHeight="1">
+    <row r="102" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A102" t="s">
         <v>580</v>
       </c>
@@ -12414,7 +12400,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="103" spans="1:24" ht="15" customHeight="1">
+    <row r="103" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A103" t="s">
         <v>580</v>
       </c>
@@ -12470,7 +12456,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="104" spans="1:24">
+    <row r="104" spans="1:24" hidden="1">
       <c r="A104" t="s">
         <v>580</v>
       </c>
@@ -12526,7 +12512,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="105" spans="1:24" ht="15" customHeight="1">
+    <row r="105" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A105" t="s">
         <v>580</v>
       </c>
@@ -12582,7 +12568,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="106" spans="1:24" ht="15" customHeight="1">
+    <row r="106" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A106" t="s">
         <v>580</v>
       </c>
@@ -12638,7 +12624,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="107" spans="1:24" ht="15" customHeight="1">
+    <row r="107" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A107" s="7" t="s">
         <v>712</v>
       </c>
@@ -12710,7 +12696,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="108" spans="1:24" ht="15" customHeight="1">
+    <row r="108" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A108" s="7" t="s">
         <v>712</v>
       </c>
@@ -12782,7 +12768,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="109" spans="1:24" ht="15" customHeight="1">
+    <row r="109" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A109" t="s">
         <v>712</v>
       </c>
@@ -12853,7 +12839,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="110" spans="1:24" ht="15" customHeight="1">
+    <row r="110" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A110" s="7" t="s">
         <v>712</v>
       </c>
@@ -12916,7 +12902,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="111" spans="1:24">
+    <row r="111" spans="1:24" hidden="1">
       <c r="A111" s="7" t="s">
         <v>712</v>
       </c>
@@ -12988,7 +12974,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="112" spans="1:24" ht="15" customHeight="1">
+    <row r="112" spans="1:24" ht="15" hidden="1" customHeight="1">
       <c r="A112" s="7" t="s">
         <v>712</v>
       </c>
@@ -13060,7 +13046,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="113" spans="1:32" ht="15" customHeight="1">
+    <row r="113" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A113" s="7" t="s">
         <v>712</v>
       </c>
@@ -13071,7 +13057,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="114" spans="1:32" ht="15" customHeight="1">
+    <row r="114" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A114" s="7" t="s">
         <v>712</v>
       </c>
@@ -13082,7 +13068,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="115" spans="1:32" ht="15" customHeight="1">
+    <row r="115" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A115" s="7" t="s">
         <v>712</v>
       </c>
@@ -13165,7 +13151,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="117" spans="1:32" ht="15" customHeight="1">
+    <row r="117" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A117" s="7" t="s">
         <v>760</v>
       </c>
@@ -13237,7 +13223,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="118" spans="1:32" ht="15" customHeight="1">
+    <row r="118" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A118" s="7" t="s">
         <v>760</v>
       </c>
@@ -13309,7 +13295,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="119" spans="1:32" ht="15" customHeight="1">
+    <row r="119" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A119" s="7" t="s">
         <v>760</v>
       </c>
@@ -13453,7 +13439,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="121" spans="1:32" ht="15" customHeight="1">
+    <row r="121" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A121" s="7" t="s">
         <v>785</v>
       </c>
@@ -13597,7 +13583,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="123" spans="1:32" ht="15" customHeight="1">
+    <row r="123" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A123" s="7" t="s">
         <v>799</v>
       </c>
@@ -13669,7 +13655,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="124" spans="1:32" ht="15" customHeight="1">
+    <row r="124" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A124" s="7" t="s">
         <v>799</v>
       </c>
@@ -13741,7 +13727,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="125" spans="1:32" ht="15" customHeight="1">
+    <row r="125" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A125" s="7" t="s">
         <v>799</v>
       </c>
@@ -13752,7 +13738,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="126" spans="1:32" ht="15" customHeight="1">
+    <row r="126" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A126" t="s">
         <v>820</v>
       </c>
@@ -13824,7 +13810,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="127" spans="1:32" ht="15" customHeight="1">
+    <row r="127" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A127" t="s">
         <v>820</v>
       </c>
@@ -13896,7 +13882,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="128" spans="1:32" ht="15" customHeight="1">
+    <row r="128" spans="1:32" ht="15" hidden="1" customHeight="1">
       <c r="A128" t="s">
         <v>820</v>
       </c>
@@ -13975,6 +13961,10 @@
       <c r="AE128" s="7"/>
       <c r="AF128" s="7"/>
     </row>
+    <row r="129" ht="15" hidden="1" customHeight="1"/>
+    <row r="130" ht="15" hidden="1" customHeight="1"/>
+    <row r="131" ht="15" hidden="1" customHeight="1"/>
+    <row r="132" ht="15" hidden="1" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="F61:F62">
     <cfRule type="expression" dxfId="42" priority="13">
@@ -14158,10 +14148,13 @@
     <hyperlink ref="F5" r:id="rId165" xr:uid="{4A3391DB-DBED-4F3C-AFE8-623EA0388EFE}"/>
     <hyperlink ref="F118" r:id="rId166" xr:uid="{FF1F9950-9EBB-4A48-BDA7-40BC8F0F30B9}"/>
     <hyperlink ref="F112" r:id="rId167" xr:uid="{BEBDBF27-15FA-4171-B9BB-AEB9EE1C5693}"/>
+    <hyperlink ref="O72" r:id="rId168" xr:uid="{6AB0B00B-BE9B-488B-ACF2-75D827FF2BAF}"/>
+    <hyperlink ref="O3" r:id="rId169" xr:uid="{8BBAF721-9ABD-42B2-98E0-F51D8D8C3E35}"/>
+    <hyperlink ref="O54" r:id="rId170" xr:uid="{347D6AAE-AE93-49E9-982A-04E82CB14A4E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId168"/>
+    <tablePart r:id="rId171"/>
   </tableParts>
 </worksheet>
 </file>
@@ -20564,10 +20557,10 @@
         <v>8</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>347</v>
+        <v>1283</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -20575,10 +20568,10 @@
         <v>8</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -20589,7 +20582,7 @@
         <v>50</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>1286</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -20597,10 +20590,10 @@
         <v>8</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -20611,7 +20604,7 @@
         <v>753</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -20622,7 +20615,7 @@
         <v>32</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -20633,7 +20626,7 @@
         <v>595</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -20644,7 +20637,7 @@
         <v>648</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -20655,12 +20648,12 @@
         <v>670</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B57" s="7" t="s">
         <v>28</v>
@@ -20671,7 +20664,7 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B58" s="7" t="s">
         <v>1296</v>
@@ -20682,7 +20675,7 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B59" s="7" t="s">
         <v>41</v>
@@ -20693,7 +20686,7 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B60" s="7" t="s">
         <v>472</v>
@@ -20704,7 +20697,7 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B61" s="7" t="s">
         <v>1300</v>
@@ -20715,7 +20708,7 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B62" s="7" t="s">
         <v>1302</v>
@@ -20726,7 +20719,7 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B63" s="7" t="s">
         <v>1304</v>
@@ -20737,7 +20730,7 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B64" s="7" t="s">
         <v>1306</v>
@@ -20748,7 +20741,7 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B65" s="7" t="s">
         <v>1308</v>
@@ -20759,7 +20752,7 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B66" s="7" t="s">
         <v>1310</v>
@@ -20770,7 +20763,7 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B67" s="7" t="s">
         <v>1312</v>
@@ -20781,7 +20774,7 @@
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B68" s="7" t="s">
         <v>1314</v>
@@ -20792,7 +20785,7 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>1294</v>
+        <v>11</v>
       </c>
       <c r="B69" s="7" t="s">
         <v>1259</v>

</xml_diff>